<commit_message>
-se hicieron graficos en excel para comparar las rubricas de funcionalida y mantenibilidad
</commit_message>
<xml_diff>
--- a/metricas_realizadas/SOA/Analisis Metricas SOA/Resultados ESP32 uso CPU y memoria.xlsx
+++ b/metricas_realizadas/SOA/Analisis Metricas SOA/Resultados ESP32 uso CPU y memoria.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyecto_code_ia\metricas_realizadas\SOA\Analisis Metricas SOA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D0682A9-6EA7-4B84-9360-D97EF3D1B005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3DC0C37-3A50-47BD-8549-DD8B178385FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -467,14 +467,14 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3388,14 +3388,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
@@ -3441,7 +3441,7 @@
       <c r="A4" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="16">
+      <c r="B4" s="15">
         <v>8.9600000000000009</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -3546,14 +3546,14 @@
       <c r="F9" s="3"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
@@ -3668,10 +3668,10 @@
       <c r="D17" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="E17" s="17">
+      <c r="E17" s="16">
         <v>16.239999999999998</v>
       </c>
-      <c r="F17" s="17" t="s">
+      <c r="F17" s="16" t="s">
         <v>73</v>
       </c>
     </row>
@@ -3734,12 +3734,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
       <c r="E1" s="14"/>
       <c r="F1" s="14"/>
       <c r="G1" s="9"/>
@@ -3850,12 +3850,12 @@
       <c r="D9" s="3"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
     </row>

</xml_diff>